<commit_message>
Update model outputs 2026-07-01 14:18:11
</commit_message>
<xml_diff>
--- a/files/SSN_upcoming_projections.xlsx
+++ b/files/SSN_upcoming_projections.xlsx
@@ -65,10 +65,10 @@
     <t xml:space="preserve">1H</t>
   </si>
   <si>
+    <t xml:space="preserve">Adelaide Thunderbirds</t>
+  </si>
+  <si>
     <t xml:space="preserve">Melbourne Vixens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">West Coast Fever</t>
   </si>
   <si>
     <t xml:space="preserve">1Q</t>
@@ -411,7 +411,7 @@
   <cols>
     <col min="1" max="1" width="11.2056266178838" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="15.8703495591654" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="16.7099996885961" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="21.7099995912824" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="16.7099996885961" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.704168823845" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="15.8703495591654" hidden="0" customWidth="1"/>
@@ -479,7 +479,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46200</v>
+        <v>46207</v>
       </c>
       <c r="B2" t="s">
         <v>16</v>
@@ -491,45 +491,45 @@
         <v>18</v>
       </c>
       <c r="E2" t="n">
-        <v>0.35</v>
+        <v>-5.36</v>
       </c>
       <c r="F2" t="n">
-        <v>59.34</v>
+        <v>52.78</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.28</v>
+        <v>-0.27</v>
       </c>
       <c r="H2" t="n">
-        <v>0.35</v>
+        <v>-5.48</v>
       </c>
       <c r="I2" t="n">
-        <v>58.15</v>
+        <v>54.39</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>0.86</v>
+        <v>1.06</v>
       </c>
       <c r="L2" t="n">
-        <v>0.8</v>
+        <v>1.07</v>
       </c>
       <c r="M2" t="n">
-        <v>0.24</v>
+        <v>0.18</v>
       </c>
       <c r="N2" t="n">
-        <v>-0.19</v>
+        <v>0.25</v>
       </c>
       <c r="O2" t="n">
-        <v>0.59</v>
+        <v>-5.18</v>
       </c>
       <c r="P2" t="n">
-        <v>59.15</v>
+        <v>53.03</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46200</v>
+        <v>46207</v>
       </c>
       <c r="B3" t="s">
         <v>19</v>
@@ -541,45 +541,45 @@
         <v>18</v>
       </c>
       <c r="E3" t="n">
-        <v>0.14</v>
+        <v>-2.25</v>
       </c>
       <c r="F3" t="n">
-        <v>30.02</v>
+        <v>26.7</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.28</v>
+        <v>-0.27</v>
       </c>
       <c r="H3" t="n">
-        <v>0.15</v>
+        <v>-2.3</v>
       </c>
       <c r="I3" t="n">
-        <v>29.42</v>
+        <v>27.51</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>0.86</v>
+        <v>1.06</v>
       </c>
       <c r="L3" t="n">
-        <v>0.8</v>
+        <v>1.07</v>
       </c>
       <c r="M3" t="n">
-        <v>0.12</v>
+        <v>0.09</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.1</v>
+        <v>0.13</v>
       </c>
       <c r="O3" t="n">
-        <v>0.27</v>
+        <v>-2.16</v>
       </c>
       <c r="P3" t="n">
-        <v>29.92</v>
+        <v>26.83</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46200</v>
+        <v>46207</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
@@ -591,40 +591,40 @@
         <v>18</v>
       </c>
       <c r="E4" t="n">
-        <v>0.67</v>
+        <v>-10.38</v>
       </c>
       <c r="F4" t="n">
-        <v>117.88</v>
+        <v>104.85</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.28</v>
+        <v>-0.27</v>
       </c>
       <c r="H4" t="n">
-        <v>0.68</v>
+        <v>-10.62</v>
       </c>
       <c r="I4" t="n">
-        <v>115.51</v>
+        <v>108.04</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0.86</v>
+        <v>1.06</v>
       </c>
       <c r="L4" t="n">
-        <v>0.8</v>
+        <v>1.07</v>
       </c>
       <c r="M4" t="n">
-        <v>0.48</v>
+        <v>0.36</v>
       </c>
       <c r="N4" t="n">
-        <v>-0.38</v>
+        <v>0.5</v>
       </c>
       <c r="O4" t="n">
-        <v>1.15</v>
+        <v>-10.02</v>
       </c>
       <c r="P4" t="n">
-        <v>117.49</v>
+        <v>105.35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>